<commit_message>
Weekly portfolio data update (2026-08-17)
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="13680" yWindow="1940" windowWidth="20520" windowHeight="16920" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="History" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="History" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="181029" fullCalcOnLoad="1"/>
@@ -539,6 +539,9 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="5" t="inlineStr">
         <is>
@@ -604,7 +607,7 @@
         <v>41.5</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>35.83</v>
+        <v>31.88</v>
       </c>
       <c r="G6" s="6">
         <f>(F6-E6)/E6</f>
@@ -615,7 +618,7 @@
         <v/>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.0352</v>
+        <v>0.0389</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -641,7 +644,7 @@
         <v>25.6</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>28.36</v>
+        <v>30.95</v>
       </c>
       <c r="G7" s="7">
         <f>(F7-E7)/E7</f>
@@ -652,7 +655,7 @@
         <v/>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.0387</v>
+        <v>0.0423</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -678,7 +681,7 @@
         <v>38</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>35.99</v>
+        <v>38.97</v>
       </c>
       <c r="G8" s="6">
         <f>(F8-E8)/E8</f>
@@ -689,7 +692,7 @@
         <v/>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.0381</v>
+        <v>0.0421</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -715,7 +718,7 @@
         <v>14.67</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>15.98</v>
+        <v>16.7</v>
       </c>
       <c r="G9" s="7">
         <f>(F9-E9)/E9</f>
@@ -726,7 +729,7 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.1008</v>
+        <v>0.1126</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -734,6 +737,9 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13" ht="21" customHeight="1" s="11" thickBot="1">
       <c r="B13" s="8" t="inlineStr">
         <is>
@@ -805,7 +811,9 @@
       <c r="F16" s="13" t="n">
         <v>3.72</v>
       </c>
-      <c r="G16" s="3" t="n"/>
+      <c r="G16" s="3" t="n">
+        <v>3.06</v>
+      </c>
       <c r="H16" s="3" t="n"/>
       <c r="I16" s="13">
         <f>E16+F16</f>
@@ -833,6 +841,9 @@
       <c r="F17" s="13" t="n">
         <v>2.5</v>
       </c>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
       <c r="I17" s="13">
         <f>E17+F17</f>
         <v/>
@@ -859,6 +870,9 @@
       <c r="F18" s="13" t="n">
         <v>2.7</v>
       </c>
+      <c r="G18" t="n">
+        <v>5.39</v>
+      </c>
       <c r="I18" s="13">
         <f>E18+F18</f>
         <v/>
@@ -884,6 +898,9 @@
       </c>
       <c r="F19" s="15" t="n">
         <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1.41</v>
       </c>
       <c r="I19" s="13">
         <f>E19+F19</f>
@@ -914,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -969,6 +986,142 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AD:AMS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Ahold</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" t="n">
+        <v>31.88</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0.0389</v>
+      </c>
+      <c r="H2" t="n">
+        <v>191.28</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ING:AMS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ING</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>30.95</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0.0423</v>
+      </c>
+      <c r="H3" t="n">
+        <v>154.77</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SHELL:AMS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>38.97</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0421</v>
+      </c>
+      <c r="H4" t="n">
+        <v>311.8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HTGC:NYSE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>0.1126</v>
+      </c>
+      <c r="H5" t="n">
+        <v>50.1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly portfolio data update (2026-08-24)
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -607,7 +607,7 @@
         <v>41.5</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>31.88</v>
+        <v>31.04</v>
       </c>
       <c r="G6" s="6">
         <f>(F6-E6)/E6</f>
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.0389</v>
+        <v>0.0399</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         <v>25.6</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>30.95</v>
+        <v>29.83</v>
       </c>
       <c r="G7" s="7">
         <f>(F7-E7)/E7</f>
@@ -655,7 +655,7 @@
         <v/>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.0423</v>
+        <v>0.0438</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
         <v>38</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>38.97</v>
+        <v>39.91</v>
       </c>
       <c r="G8" s="6">
         <f>(F8-E8)/E8</f>
@@ -692,7 +692,7 @@
         <v/>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.0421</v>
+        <v>0.0408</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>14.67</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>16.7</v>
+        <v>17.13</v>
       </c>
       <c r="G9" s="7">
         <f>(F9-E9)/E9</f>
@@ -729,7 +729,7 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.1126</v>
+        <v>0.1097</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         <v>2.7</v>
       </c>
       <c r="G18" t="n">
-        <v>5.39</v>
+        <v>5.35</v>
       </c>
       <c r="I18" s="13">
         <f>E18+F18</f>
@@ -931,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -1122,6 +1122,142 @@
         <v>50.1</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AD:AMS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Ahold</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>31.04</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>0.0399</v>
+      </c>
+      <c r="H6" t="n">
+        <v>186.24</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ING:AMS</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ING</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>29.83</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0.0438</v>
+      </c>
+      <c r="H7" t="n">
+        <v>149.15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SHELL:AMS</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>39.91</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>0.0408</v>
+      </c>
+      <c r="H8" t="n">
+        <v>319.28</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HTGC:NYSE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>17.13</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>0.1097</v>
+      </c>
+      <c r="H9" t="n">
+        <v>51.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly portfolio data update (2026-08-31)
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -607,7 +607,7 @@
         <v>41.5</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>31.04</v>
+        <v>30.54</v>
       </c>
       <c r="G6" s="6">
         <f>(F6-E6)/E6</f>
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.0399</v>
+        <v>0.0406</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         <v>25.6</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>29.83</v>
+        <v>30.59</v>
       </c>
       <c r="G7" s="7">
         <f>(F7-E7)/E7</f>
@@ -655,7 +655,7 @@
         <v/>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.0438</v>
+        <v>0.0428</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
         <v>38</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>39.91</v>
+        <v>39.58</v>
       </c>
       <c r="G8" s="6">
         <f>(F8-E8)/E8</f>
@@ -692,7 +692,7 @@
         <v/>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.0408</v>
+        <v>0.0414</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>14.67</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>17.13</v>
+        <v>17.48</v>
       </c>
       <c r="G9" s="7">
         <f>(F9-E9)/E9</f>
@@ -729,7 +729,7 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.1097</v>
+        <v>0.1076</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         <v>2.7</v>
       </c>
       <c r="G18" t="n">
-        <v>5.35</v>
+        <v>5.38</v>
       </c>
       <c r="I18" s="13">
         <f>E18+F18</f>
@@ -931,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -1258,6 +1258,142 @@
         <v>51.39</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AD:AMS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ahold</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" t="n">
+        <v>30.54</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0.0406</v>
+      </c>
+      <c r="H10" t="n">
+        <v>183.24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ING:AMS</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ING</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>30.59</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>0.0428</v>
+      </c>
+      <c r="H11" t="n">
+        <v>152.95</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SHELL:AMS</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" t="n">
+        <v>39.58</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>0.0414</v>
+      </c>
+      <c r="H12" t="n">
+        <v>316.68</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HTGC:NYSE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>17.48</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>0.1076</v>
+      </c>
+      <c r="H13" t="n">
+        <v>52.44</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Weekly portfolio data update (2026-09-07)
</commit_message>
<xml_diff>
--- a/data/portfolio.xlsx
+++ b/data/portfolio.xlsx
@@ -607,7 +607,7 @@
         <v>41.5</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>30.54</v>
+        <v>31.39</v>
       </c>
       <c r="G6" s="6">
         <f>(F6-E6)/E6</f>
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="I6" s="4" t="n">
-        <v>0.0406</v>
+        <v>0.0395</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -644,7 +644,7 @@
         <v>25.6</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>30.59</v>
+        <v>32.04</v>
       </c>
       <c r="G7" s="7">
         <f>(F7-E7)/E7</f>
@@ -655,7 +655,7 @@
         <v/>
       </c>
       <c r="I7" s="4" t="n">
-        <v>0.0428</v>
+        <v>0.0408</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -681,7 +681,7 @@
         <v>38</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>39.58</v>
+        <v>40.49</v>
       </c>
       <c r="G8" s="6">
         <f>(F8-E8)/E8</f>
@@ -692,7 +692,7 @@
         <v/>
       </c>
       <c r="I8" s="4" t="n">
-        <v>0.0414</v>
+        <v>0.0404</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -718,7 +718,7 @@
         <v>14.67</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>17.48</v>
+        <v>17.63</v>
       </c>
       <c r="G9" s="7">
         <f>(F9-E9)/E9</f>
@@ -729,7 +729,7 @@
         <v/>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0.1076</v>
+        <v>0.1066</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -931,7 +931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -1394,6 +1394,142 @@
         <v>52.44</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>AD:AMS</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ahold</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" t="n">
+        <v>31.39</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>0.0395</v>
+      </c>
+      <c r="H14" t="n">
+        <v>188.34</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ING:AMS</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ING</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>32.04</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>0.0408</v>
+      </c>
+      <c r="H15" t="n">
+        <v>160.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SHELL:AMS</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Shell</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" t="n">
+        <v>40.49</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>0.0404</v>
+      </c>
+      <c r="H16" t="n">
+        <v>323.88</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HTGC:NYSE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>17.63</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>0.1066</v>
+      </c>
+      <c r="H17" t="n">
+        <v>52.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>